<commit_message>
start cleaning according to new rules
</commit_message>
<xml_diff>
--- a/Rule 10.2.2026.xlsx
+++ b/Rule 10.2.2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OS TDTS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\estates-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC6D83AC-1B12-4AFE-90C5-A2742A44F225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAC4623D-885C-4CB1-8421-9A5F3D4CFB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14460" yWindow="0" windowWidth="14445" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rule dat - BDS.com" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="114">
   <si>
     <t>STT</t>
   </si>
@@ -992,6 +992,9 @@
   </si>
   <si>
     <t>Cần bổ sung phần scrape biệt thự, shophouse.</t>
+  </si>
+  <si>
+    <t>dtxd, diện tích xây dựng, dt xây dựng, diện tích xd, (có thể thôi, phải check lại) xây dựng \d+\s*m, xd \d+\s*m</t>
   </si>
 </sst>
 </file>
@@ -1038,12 +1041,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -1073,7 +1082,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1143,11 +1152,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1891,17 +1912,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D996C110-4D1D-4AE6-94B9-25638ED611BF}">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
     <col min="2" max="2" width="24.5703125" style="7" customWidth="1"/>
     <col min="3" max="3" width="49.85546875" style="7" customWidth="1"/>
-    <col min="4" max="4" width="96.5703125" style="7" customWidth="1"/>
-    <col min="5" max="5" width="80.5703125" style="19" customWidth="1"/>
+    <col min="4" max="4" width="73.28515625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="73.28515625" style="19" customWidth="1"/>
+    <col min="6" max="6" width="27.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -1918,7 +1940,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1930,8 +1952,9 @@
       </c>
       <c r="D2" s="10"/>
       <c r="E2" s="20"/>
-    </row>
-    <row r="3" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="F2" s="6"/>
+    </row>
+    <row r="3" spans="1:6" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -1943,8 +1966,9 @@
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="21"/>
-    </row>
-    <row r="4" spans="1:5" s="9" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F3" s="25"/>
+    </row>
+    <row r="4" spans="1:6" s="9" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -1956,8 +1980,9 @@
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="21"/>
-    </row>
-    <row r="5" spans="1:5" s="9" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F4" s="25"/>
+    </row>
+    <row r="5" spans="1:6" s="9" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -1971,8 +1996,9 @@
         <v>35</v>
       </c>
       <c r="E5" s="21"/>
-    </row>
-    <row r="6" spans="1:5" s="9" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F5" s="25"/>
+    </row>
+    <row r="6" spans="1:6" s="9" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -1986,8 +2012,9 @@
         <v>36</v>
       </c>
       <c r="E6" s="21"/>
-    </row>
-    <row r="7" spans="1:5" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F6" s="25"/>
+    </row>
+    <row r="7" spans="1:6" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -1999,8 +2026,9 @@
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="21"/>
-    </row>
-    <row r="8" spans="1:5" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F7" s="25"/>
+    </row>
+    <row r="8" spans="1:6" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -2012,8 +2040,9 @@
       </c>
       <c r="D8" s="10"/>
       <c r="E8" s="21"/>
-    </row>
-    <row r="9" spans="1:5" s="9" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F8" s="25"/>
+    </row>
+    <row r="9" spans="1:6" s="9" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -2025,23 +2054,25 @@
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="21"/>
-    </row>
-    <row r="10" spans="1:5" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F9" s="25"/>
+    </row>
+    <row r="10" spans="1:6" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="25" t="s">
+      <c r="D10" s="26"/>
+      <c r="E10" s="27" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F10" s="25"/>
+    </row>
+    <row r="11" spans="1:6" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -2053,8 +2084,9 @@
       </c>
       <c r="D11" s="10"/>
       <c r="E11" s="21"/>
-    </row>
-    <row r="12" spans="1:5" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F11" s="25"/>
+    </row>
+    <row r="12" spans="1:6" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -2066,8 +2098,9 @@
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="21"/>
-    </row>
-    <row r="13" spans="1:5" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F12" s="25"/>
+    </row>
+    <row r="13" spans="1:6" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -2079,8 +2112,9 @@
       </c>
       <c r="D13" s="10"/>
       <c r="E13" s="21"/>
-    </row>
-    <row r="14" spans="1:5" s="9" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F13" s="25"/>
+    </row>
+    <row r="14" spans="1:6" s="9" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -2094,8 +2128,9 @@
         <v>45</v>
       </c>
       <c r="E14" s="21"/>
-    </row>
-    <row r="15" spans="1:5" s="9" customFormat="1" ht="262.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F14" s="25"/>
+    </row>
+    <row r="15" spans="1:6" s="9" customFormat="1" ht="262.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -2109,8 +2144,9 @@
         <v>47</v>
       </c>
       <c r="E15" s="21"/>
-    </row>
-    <row r="16" spans="1:5" s="9" customFormat="1" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F15" s="25"/>
+    </row>
+    <row r="16" spans="1:6" s="9" customFormat="1" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -2124,42 +2160,47 @@
         <v>74</v>
       </c>
       <c r="E16" s="21"/>
-    </row>
-    <row r="17" spans="1:5" s="9" customFormat="1" ht="153.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="5">
+      <c r="F16" s="25"/>
+    </row>
+    <row r="17" spans="1:6" s="9" customFormat="1" ht="153.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="28">
         <v>16</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="22" t="s">
+      <c r="E17" s="29" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" s="9" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="5">
+      <c r="F17" s="25" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="9" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="28">
         <v>17</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="29" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" s="9" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F18" s="25"/>
+    </row>
+    <row r="19" spans="1:6" s="9" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -2171,8 +2212,9 @@
       </c>
       <c r="D19" s="10"/>
       <c r="E19" s="21"/>
-    </row>
-    <row r="20" spans="1:5" s="9" customFormat="1" ht="234.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F19" s="25"/>
+    </row>
+    <row r="20" spans="1:6" s="9" customFormat="1" ht="234.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -2186,8 +2228,9 @@
         <v>78</v>
       </c>
       <c r="E20" s="21"/>
-    </row>
-    <row r="21" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="F20" s="25"/>
+    </row>
+    <row r="21" spans="1:6" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -2199,8 +2242,9 @@
       </c>
       <c r="D21" s="10"/>
       <c r="E21" s="21"/>
-    </row>
-    <row r="22" spans="1:5" s="9" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="F21" s="25"/>
+    </row>
+    <row r="22" spans="1:6" s="9" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -2214,8 +2258,9 @@
         <v>51</v>
       </c>
       <c r="E22" s="21"/>
-    </row>
-    <row r="23" spans="1:5" s="9" customFormat="1" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F22" s="25"/>
+    </row>
+    <row r="23" spans="1:6" s="9" customFormat="1" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -2229,8 +2274,9 @@
         <v>53</v>
       </c>
       <c r="E23" s="21"/>
-    </row>
-    <row r="24" spans="1:5" s="9" customFormat="1" ht="111" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F23" s="25"/>
+    </row>
+    <row r="24" spans="1:6" s="9" customFormat="1" ht="111" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -2244,8 +2290,9 @@
         <v>55</v>
       </c>
       <c r="E24" s="21"/>
-    </row>
-    <row r="25" spans="1:5" s="9" customFormat="1" ht="232.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F24" s="25"/>
+    </row>
+    <row r="25" spans="1:6" s="9" customFormat="1" ht="232.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>24</v>
       </c>
@@ -2259,59 +2306,63 @@
         <v>57</v>
       </c>
       <c r="E25" s="21"/>
-    </row>
-    <row r="26" spans="1:5" s="9" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="5">
+      <c r="F25" s="25"/>
+    </row>
+    <row r="26" spans="1:6" s="9" customFormat="1" ht="255" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="28">
         <v>25</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="22" t="s">
+      <c r="E26" s="29" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" s="9" customFormat="1" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="5">
+      <c r="F26" s="25"/>
+    </row>
+    <row r="27" spans="1:6" s="9" customFormat="1" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="28">
         <v>26</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="E27" s="22" t="s">
+      <c r="E27" s="29" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" s="9" customFormat="1" ht="195" x14ac:dyDescent="0.25">
-      <c r="A28" s="5">
+      <c r="F27" s="25"/>
+    </row>
+    <row r="28" spans="1:6" s="9" customFormat="1" ht="210" x14ac:dyDescent="0.25">
+      <c r="A28" s="28">
         <v>27</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="E28" s="23" t="s">
+      <c r="E28" s="30" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" s="9" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F28" s="25"/>
+    </row>
+    <row r="29" spans="1:6" s="9" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>28</v>
       </c>
@@ -2323,8 +2374,9 @@
       </c>
       <c r="D29" s="10"/>
       <c r="E29" s="21"/>
-    </row>
-    <row r="30" spans="1:5" s="9" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F29" s="25"/>
+    </row>
+    <row r="30" spans="1:6" s="9" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>29</v>
       </c>
@@ -2336,8 +2388,9 @@
       </c>
       <c r="D30" s="10"/>
       <c r="E30" s="21"/>
-    </row>
-    <row r="31" spans="1:5" s="9" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F30" s="25"/>
+    </row>
+    <row r="31" spans="1:6" s="9" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>30</v>
       </c>
@@ -2349,6 +2402,7 @@
       </c>
       <c r="D31" s="10"/>
       <c r="E31" s="21"/>
+      <c r="F31" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2624,7 +2678,7 @@
       <c r="E18" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="F18" s="26" t="s">
+      <c r="F18" s="25" t="s">
         <v>111</v>
       </c>
     </row>
@@ -2655,7 +2709,7 @@
       <c r="E20" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="F20" s="26" t="s">
+      <c r="F20" s="25" t="s">
         <v>112</v>
       </c>
     </row>

</xml_diff>

<commit_message>
started changing rules for tong dien tich san
</commit_message>
<xml_diff>
--- a/Rule 10.2.2026.xlsx
+++ b/Rule 10.2.2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\estates-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAC4623D-885C-4CB1-8421-9A5F3D4CFB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5833B72B-172D-4C24-9963-4ACB07AF7CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14460" yWindow="0" windowWidth="14445" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rule dat - BDS.com" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="115">
   <si>
     <t>STT</t>
   </si>
@@ -995,6 +995,57 @@
   </si>
   <si>
     <t>dtxd, diện tích xây dựng, dt xây dựng, diện tích xd, (có thể thôi, phải check lại) xây dựng \d+\s*m, xd \d+\s*m</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Nếu trích xuất được các cụm </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>diện tích sàn, diện tích sử dụng</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> thì sẽ lưu nó thành tổng diện tích sàn
+Nếu không có những cụm trên, tổng diện tích sàn sẽ được tính bằng diện tích xây dựng * tổng số tầng công trình. Diện tích xây dựng được xác định như sau:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Nếu có "diện tích xây dựng" trên đất là bao nhiêu m2 thì trả về đúng giá trị đó</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- Nếu có các cụm thổ cư / đất ở bao nhiêu m thì trả về giá trị xây dựng bằng giá trị được viết ở đây
+- Nếu không có các giá trị ở trên, mặc định diện tích xây dựng = diện tích đất</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2176,7 +2227,7 @@
         <v>48</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="F17" s="25" t="s">
         <v>113</v>

</xml_diff>